<commit_message>
xlstream-eval: consolidate cross-sheet tests into conformance fixture
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/issues/issue-136-cross-sheet-cell-ref.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/issues/issue-136-cross-sheet-cell-ref.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-cross-sheet-cell-ref/crates/xlstream-eval/tests/fixtures/issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_25F82EEB8B4CD0E975A607F620BB4211A74A43A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_BD8B1C4F324E5C2B1CB07623269B5C62E9C7F0A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Tax Rates" sheetId="4" r:id="rId4"/>
+    <sheet name="Rates" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Input</t>
   </si>
@@ -52,6 +55,18 @@
   </si>
   <si>
     <t>Concat</t>
+  </si>
+  <si>
+    <t>SelfRef</t>
+  </si>
+  <si>
+    <t>SelfPlusCross</t>
+  </si>
+  <si>
+    <t>MultiSheet</t>
+  </si>
+  <si>
+    <t>QuotedSheet</t>
   </si>
   <si>
     <t>hello</t>
@@ -397,10 +412,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -419,8 +434,20 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>10</v>
       </c>
@@ -444,8 +471,24 @@
         <f>CONCATENATE("x",Sheet2!D1)</f>
         <v>xhello</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2">
+        <f>Sheet1!A2*2</f>
+        <v>20</v>
+      </c>
+      <c r="H2">
+        <f>Sheet2!A1+Sheet1!A2</f>
+        <v>110</v>
+      </c>
+      <c r="I2">
+        <f>Sheet2!A1+Sheet3!A1</f>
+        <v>150</v>
+      </c>
+      <c r="J2">
+        <f>A2*'Tax Rates'!A1</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0</v>
       </c>
@@ -468,6 +511,31 @@
       <c r="F3" t="str">
         <f>CONCATENATE("y",Sheet2!D2)</f>
         <v>yworld</v>
+      </c>
+      <c r="G3">
+        <f>Sheet1!A3*2</f>
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <f>Sheet2!A1+Sheet1!A3</f>
+        <v>100</v>
+      </c>
+      <c r="I3">
+        <f>IF(A3&gt;0,Sheet2!A1,Sheet3!A1)</f>
+        <v>50</v>
+      </c>
+      <c r="J3">
+        <f>A3*'Tax Rates'!A1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <f>A4*Rates!A2</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -491,7 +559,7 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -505,7 +573,57 @@
         <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>0.15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>